<commit_message>
Make the examples look like Calvin's schedules
Academic year AY25, terms FA, WI, SP and SU, first and second halves of a term, a
cross-listing, non-teaching load, and a standard-times rule for the intensive terms.
The conflicts example is a small realistic schedule with a few deliberate problems.

Assisted by Claude Sonnet 5.5 (Anthropic).
</commit_message>
<xml_diff>
--- a/apps/web/public/examples/example-with-constraint-rules.xlsx
+++ b/apps/web/public/examples/example-with-constraint-rules.xlsx
@@ -391,100 +391,100 @@
     <t>EnrollmentDay10</t>
   </si>
   <si>
-    <t>R2-FA-MATH231-A</t>
-  </si>
-  <si>
-    <t>R2</t>
+    <t>AY25-FA-MATH231-A</t>
+  </si>
+  <si>
+    <t>AY25</t>
   </si>
   <si>
     <t>10:20</t>
   </si>
   <si>
-    <t>R2-FA-MATH231-B</t>
+    <t>AY25-FA-MATH231-B</t>
   </si>
   <si>
     <t>11:00</t>
   </si>
   <si>
-    <t>R2-FA-STAT243-A</t>
-  </si>
-  <si>
-    <t>R2-FA-MATH250-A</t>
+    <t>AY25-FA-STAT243-A</t>
+  </si>
+  <si>
+    <t>AY25-FA-MATH250-A</t>
   </si>
   <si>
     <t>09:15</t>
   </si>
   <si>
-    <t>R2-FA-DATA202-A</t>
-  </si>
-  <si>
-    <t>R2-FA-DATA301-A</t>
+    <t>AY25-FA-DATA202-A</t>
+  </si>
+  <si>
+    <t>AY25-FA-DATA301-A</t>
   </si>
   <si>
     <t>12:15</t>
   </si>
   <si>
-    <t>R2-FA-STAT343-A</t>
-  </si>
-  <si>
-    <t>R2-FA-CS262-A</t>
+    <t>AY25-FA-STAT343-A</t>
+  </si>
+  <si>
+    <t>AY25-FA-CS262-A</t>
   </si>
   <si>
     <t>13:30</t>
   </si>
   <si>
-    <t>R2-FA-CS108-A</t>
+    <t>AY25-FA-CS108-A</t>
   </si>
   <si>
     <t>14:45</t>
   </si>
   <si>
-    <t>R2-FA-CS372-A</t>
+    <t>AY25-FA-CS372-A</t>
   </si>
   <si>
     <t>16:00</t>
   </si>
   <si>
-    <t>R2-FA-CS108-B</t>
+    <t>AY25-FA-CS108-B</t>
   </si>
   <si>
     <t>08:00</t>
   </si>
   <si>
-    <t>R2-FA-MATH301-A</t>
+    <t>AY25-FA-MATH301-A</t>
   </si>
   <si>
     <t>14:10</t>
   </si>
   <si>
-    <t>R2-FA-MATH290-A</t>
+    <t>AY25-FA-MATH290-A</t>
   </si>
   <si>
     <t>15:05</t>
   </si>
   <si>
-    <t>R2-FA-STAT143-A</t>
-  </si>
-  <si>
-    <t>R2-FA-STAT143-B</t>
-  </si>
-  <si>
-    <t>R2-FA-STAT143-C</t>
+    <t>AY25-FA-STAT143-A</t>
+  </si>
+  <si>
+    <t>AY25-FA-STAT143-B</t>
+  </si>
+  <si>
+    <t>AY25-FA-STAT143-C</t>
   </si>
   <si>
     <t>10:30</t>
   </si>
   <si>
-    <t>R2-FA-CORE100-A</t>
-  </si>
-  <si>
-    <t>R2-FA-CORE100-B</t>
-  </si>
-  <si>
-    <t>R2-SP-MATH232-A</t>
-  </si>
-  <si>
-    <t>R2-SP-STAT244-A</t>
+    <t>AY25-FA-CORE100-A</t>
+  </si>
+  <si>
+    <t>AY25-FA-CORE100-B</t>
+  </si>
+  <si>
+    <t>AY25-SP-MATH232-A</t>
+  </si>
+  <si>
+    <t>AY25-SP-STAT244-A</t>
   </si>
   <si>
     <t>Activity</t>
@@ -799,7 +799,7 @@
     <t>Export Time</t>
   </si>
   <si>
-    <t>10:15:43</t>
+    <t>10:29:00</t>
   </si>
   <si>
     <t>Academic Year</t>
@@ -2412,7 +2412,7 @@
   <dimension ref="A1:X21"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="17" customWidth="1"/>
+    <col min="1" max="1" width="19" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
     <col min="4" max="4" width="6" customWidth="1"/>

</xml_diff>

<commit_message>
New constraint rule: Allow collisions
Assisted by Claude Sonnet 5.5 (Anthropic).
</commit_message>
<xml_diff>
--- a/apps/web/public/examples/example-with-constraint-rules.xlsx
+++ b/apps/web/public/examples/example-with-constraint-rules.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1441" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1557" uniqueCount="299">
   <si>
     <t>Term</t>
   </si>
@@ -331,6 +331,21 @@
     <t>Kim teaches three in a row on MWF</t>
   </si>
   <si>
+    <t>290</t>
+  </si>
+  <si>
+    <t>SB 123</t>
+  </si>
+  <si>
+    <t>Urban Seminar</t>
+  </si>
+  <si>
+    <t>Hal Fakename</t>
+  </si>
+  <si>
+    <t>A seminar run as a 200- and a 300-level course: same instructor, room and time; allowed by this department's rule</t>
+  </si>
+  <si>
     <t>315</t>
   </si>
   <si>
@@ -343,6 +358,15 @@
     <t>Planning Algorithms</t>
   </si>
   <si>
+    <t>390</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>The 300-level listing of the seminar; its load is counted with CRUD 290</t>
+  </si>
+  <si>
     <t>DIGI</t>
   </si>
   <si>
@@ -376,9 +400,6 @@
     <t>Ecology Core</t>
   </si>
   <si>
-    <t>Hal Fakename</t>
-  </si>
-  <si>
     <t>There is no evening section yet</t>
   </si>
   <si>
@@ -520,6 +541,12 @@
     <t>AY25-SP-BHAV226-A</t>
   </si>
   <si>
+    <t>AY25-FA-CRUD290-A</t>
+  </si>
+  <si>
+    <t>AY25-FA-CRUD390-A</t>
+  </si>
+  <si>
     <t>Activity</t>
   </si>
   <si>
@@ -745,6 +772,21 @@
     <t>AMUS 296 is meant to meet on only one of the standard days, so it is not flagged for that.</t>
   </si>
   <si>
+    <t>The seminar runs at two levels</t>
+  </si>
+  <si>
+    <t>collide</t>
+  </si>
+  <si>
+    <t>CRUD 290</t>
+  </si>
+  <si>
+    <t>CRUD 290 and CRUD 390 are one class, so they share an instructor, a room and a time on purpose.</t>
+  </si>
+  <si>
+    <t>CRUD 390</t>
+  </si>
+  <si>
     <t>Kind</t>
   </si>
   <si>
@@ -844,7 +886,7 @@
     <t>Export Time</t>
   </si>
   <si>
-    <t>08:32:09</t>
+    <t>21:03:16</t>
   </si>
   <si>
     <t>Academic Year</t>
@@ -1252,7 +1294,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R23"/>
+  <dimension ref="A1:R25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -2301,13 +2343,13 @@
         <v>22</v>
       </c>
       <c r="G19" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="H19" t="s">
+        <v>61</v>
+      </c>
+      <c r="I19" t="s">
         <v>105</v>
-      </c>
-      <c r="I19" t="s">
-        <v>106</v>
       </c>
       <c r="J19" t="s">
         <v>26</v>
@@ -2316,13 +2358,13 @@
         <v>27</v>
       </c>
       <c r="L19">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="M19" t="s">
+        <v>106</v>
+      </c>
+      <c r="N19" t="s">
         <v>107</v>
-      </c>
-      <c r="N19" t="s">
-        <v>95</v>
       </c>
       <c r="O19" t="s">
         <v>30</v>
@@ -2331,7 +2373,7 @@
         <v>31</v>
       </c>
       <c r="Q19" t="s">
-        <v>33</v>
+        <v>108</v>
       </c>
       <c r="R19" t="s">
         <v>33</v>
@@ -2342,7 +2384,7 @@
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>108</v>
+        <v>90</v>
       </c>
       <c r="C20" t="s">
         <v>109</v>
@@ -2360,10 +2402,10 @@
         <v>35</v>
       </c>
       <c r="H20" t="s">
-        <v>36</v>
+        <v>110</v>
       </c>
       <c r="I20" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="J20" t="s">
         <v>26</v>
@@ -2372,13 +2414,13 @@
         <v>27</v>
       </c>
       <c r="L20">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="M20" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="N20" t="s">
-        <v>112</v>
+        <v>95</v>
       </c>
       <c r="O20" t="s">
         <v>30</v>
@@ -2398,10 +2440,10 @@
         <v>18</v>
       </c>
       <c r="B21" t="s">
-        <v>108</v>
+        <v>90</v>
       </c>
       <c r="C21" t="s">
-        <v>60</v>
+        <v>113</v>
       </c>
       <c r="D21" t="s">
         <v>21</v>
@@ -2410,16 +2452,16 @@
         <v>22</v>
       </c>
       <c r="F21" t="s">
-        <v>22</v>
+        <v>114</v>
       </c>
       <c r="G21" t="s">
         <v>23</v>
       </c>
       <c r="H21" t="s">
-        <v>87</v>
+        <v>61</v>
       </c>
       <c r="I21" t="s">
-        <v>67</v>
+        <v>105</v>
       </c>
       <c r="J21" t="s">
         <v>26</v>
@@ -2431,10 +2473,10 @@
         <v>100</v>
       </c>
       <c r="M21" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="N21" t="s">
-        <v>63</v>
+        <v>107</v>
       </c>
       <c r="O21" t="s">
         <v>30</v>
@@ -2443,7 +2485,7 @@
         <v>31</v>
       </c>
       <c r="Q21" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="R21" t="s">
         <v>33</v>
@@ -2454,10 +2496,10 @@
         <v>18</v>
       </c>
       <c r="B22" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C22" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D22" t="s">
         <v>21</v>
@@ -2472,10 +2514,10 @@
         <v>35</v>
       </c>
       <c r="H22" t="s">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="I22" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="J22" t="s">
         <v>26</v>
@@ -2487,10 +2529,10 @@
         <v>65</v>
       </c>
       <c r="M22" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="N22" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="O22" t="s">
         <v>30</v>
@@ -2499,7 +2541,7 @@
         <v>31</v>
       </c>
       <c r="Q22" t="s">
-        <v>120</v>
+        <v>33</v>
       </c>
       <c r="R22" t="s">
         <v>33</v>
@@ -2510,13 +2552,13 @@
         <v>18</v>
       </c>
       <c r="B23" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C23" t="s">
-        <v>116</v>
+        <v>60</v>
       </c>
       <c r="D23" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="E23" t="s">
         <v>22</v>
@@ -2531,7 +2573,7 @@
         <v>87</v>
       </c>
       <c r="I23" t="s">
-        <v>117</v>
+        <v>67</v>
       </c>
       <c r="J23" t="s">
         <v>26</v>
@@ -2543,10 +2585,10 @@
         <v>100</v>
       </c>
       <c r="M23" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="N23" t="s">
-        <v>119</v>
+        <v>63</v>
       </c>
       <c r="O23" t="s">
         <v>30</v>
@@ -2555,9 +2597,121 @@
         <v>31</v>
       </c>
       <c r="Q23" t="s">
-        <v>33</v>
+        <v>122</v>
       </c>
       <c r="R23" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>18</v>
+      </c>
+      <c r="B24" t="s">
+        <v>123</v>
+      </c>
+      <c r="C24" t="s">
+        <v>124</v>
+      </c>
+      <c r="D24" t="s">
+        <v>21</v>
+      </c>
+      <c r="E24" t="s">
+        <v>22</v>
+      </c>
+      <c r="F24" t="s">
+        <v>22</v>
+      </c>
+      <c r="G24" t="s">
+        <v>35</v>
+      </c>
+      <c r="H24" t="s">
+        <v>52</v>
+      </c>
+      <c r="I24" t="s">
+        <v>125</v>
+      </c>
+      <c r="J24" t="s">
+        <v>26</v>
+      </c>
+      <c r="K24" t="s">
+        <v>27</v>
+      </c>
+      <c r="L24">
+        <v>65</v>
+      </c>
+      <c r="M24" t="s">
+        <v>126</v>
+      </c>
+      <c r="N24" t="s">
+        <v>107</v>
+      </c>
+      <c r="O24" t="s">
+        <v>30</v>
+      </c>
+      <c r="P24" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>127</v>
+      </c>
+      <c r="R24" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>18</v>
+      </c>
+      <c r="B25" t="s">
+        <v>123</v>
+      </c>
+      <c r="C25" t="s">
+        <v>124</v>
+      </c>
+      <c r="D25" t="s">
+        <v>34</v>
+      </c>
+      <c r="E25" t="s">
+        <v>22</v>
+      </c>
+      <c r="F25" t="s">
+        <v>22</v>
+      </c>
+      <c r="G25" t="s">
+        <v>23</v>
+      </c>
+      <c r="H25" t="s">
+        <v>87</v>
+      </c>
+      <c r="I25" t="s">
+        <v>125</v>
+      </c>
+      <c r="J25" t="s">
+        <v>26</v>
+      </c>
+      <c r="K25" t="s">
+        <v>27</v>
+      </c>
+      <c r="L25">
+        <v>100</v>
+      </c>
+      <c r="M25" t="s">
+        <v>126</v>
+      </c>
+      <c r="N25" t="s">
+        <v>107</v>
+      </c>
+      <c r="O25" t="s">
+        <v>30</v>
+      </c>
+      <c r="P25" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>33</v>
+      </c>
+      <c r="R25" t="s">
         <v>33</v>
       </c>
     </row>
@@ -2569,7 +2723,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:X23"/>
+  <dimension ref="A1:X25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="19" customWidth="1"/>
@@ -2598,13 +2752,13 @@
   <sheetData>
     <row r="1" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>0</v>
@@ -2628,22 +2782,22 @@
         <v>5</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>6</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="Q1" s="1" t="s">
         <v>12</v>
@@ -2652,10 +2806,10 @@
         <v>14</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="U1" s="1" t="s">
         <v>15</v>
@@ -2664,21 +2818,21 @@
         <v>16</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
     </row>
     <row r="2" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="B2" t="s">
         <v>33</v>
       </c>
       <c r="C2" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="D2" t="s">
         <v>18</v>
@@ -2711,7 +2865,7 @@
         <v>23</v>
       </c>
       <c r="N2" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="O2">
         <v>100</v>
@@ -2746,13 +2900,13 @@
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="B3" t="s">
         <v>33</v>
       </c>
       <c r="C3" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="D3" t="s">
         <v>18</v>
@@ -2785,7 +2939,7 @@
         <v>35</v>
       </c>
       <c r="N3" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="O3">
         <v>65</v>
@@ -2820,13 +2974,13 @@
     </row>
     <row r="4" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="B4" t="s">
         <v>33</v>
       </c>
       <c r="C4" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="D4" t="s">
         <v>18</v>
@@ -2859,7 +3013,7 @@
         <v>23</v>
       </c>
       <c r="N4" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="O4">
         <v>100</v>
@@ -2894,13 +3048,13 @@
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="B5" t="s">
         <v>33</v>
       </c>
       <c r="C5" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="D5" t="s">
         <v>18</v>
@@ -2933,7 +3087,7 @@
         <v>35</v>
       </c>
       <c r="N5" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="O5">
         <v>65</v>
@@ -2968,13 +3122,13 @@
     </row>
     <row r="6" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>148</v>
+      </c>
+      <c r="B6" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" t="s">
         <v>141</v>
-      </c>
-      <c r="B6" t="s">
-        <v>33</v>
-      </c>
-      <c r="C6" t="s">
-        <v>134</v>
       </c>
       <c r="D6" t="s">
         <v>18</v>
@@ -2983,16 +3137,16 @@
         <v>26</v>
       </c>
       <c r="F6" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="G6" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="H6" t="s">
         <v>21</v>
       </c>
       <c r="I6" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="J6">
         <v>4</v>
@@ -3007,16 +3161,16 @@
         <v>35</v>
       </c>
       <c r="N6" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="O6">
         <v>65</v>
       </c>
       <c r="P6" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="Q6" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="R6" t="s">
         <v>30</v>
@@ -3042,13 +3196,13 @@
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="B7" t="s">
         <v>33</v>
       </c>
       <c r="C7" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="D7" t="s">
         <v>18</v>
@@ -3057,7 +3211,7 @@
         <v>26</v>
       </c>
       <c r="F7" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="G7" t="s">
         <v>60</v>
@@ -3081,7 +3235,7 @@
         <v>23</v>
       </c>
       <c r="N7" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="O7">
         <v>100</v>
@@ -3090,7 +3244,7 @@
         <v>67</v>
       </c>
       <c r="Q7" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="R7" t="s">
         <v>30</v>
@@ -3105,7 +3259,7 @@
         <v>31</v>
       </c>
       <c r="V7" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="W7" t="s">
         <v>33</v>
@@ -3116,13 +3270,13 @@
     </row>
     <row r="8" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="B8" t="s">
         <v>33</v>
       </c>
       <c r="C8" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="D8" t="s">
         <v>18</v>
@@ -3155,7 +3309,7 @@
         <v>23</v>
       </c>
       <c r="N8" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="O8">
         <v>100</v>
@@ -3190,13 +3344,13 @@
     </row>
     <row r="9" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="B9" t="s">
         <v>33</v>
       </c>
       <c r="C9" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="D9" t="s">
         <v>18</v>
@@ -3229,7 +3383,7 @@
         <v>35</v>
       </c>
       <c r="N9" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="O9">
         <v>65</v>
@@ -3264,13 +3418,13 @@
     </row>
     <row r="10" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="B10" t="s">
         <v>33</v>
       </c>
       <c r="C10" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="D10" t="s">
         <v>18</v>
@@ -3303,7 +3457,7 @@
         <v>35</v>
       </c>
       <c r="N10" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="O10">
         <v>65</v>
@@ -3338,13 +3492,13 @@
     </row>
     <row r="11" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="B11" t="s">
         <v>33</v>
       </c>
       <c r="C11" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="D11" t="s">
         <v>18</v>
@@ -3356,7 +3510,7 @@
         <v>90</v>
       </c>
       <c r="G11" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="H11" t="s">
         <v>21</v>
@@ -3377,16 +3531,16 @@
         <v>35</v>
       </c>
       <c r="N11" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="O11">
         <v>60</v>
       </c>
       <c r="P11" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="Q11" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="R11" t="s">
         <v>30</v>
@@ -3412,13 +3566,13 @@
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="B12" t="s">
         <v>33</v>
       </c>
       <c r="C12" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="D12" t="s">
         <v>18</v>
@@ -3451,7 +3605,7 @@
         <v>35</v>
       </c>
       <c r="N12" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="O12">
         <v>65</v>
@@ -3486,13 +3640,13 @@
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="B13" t="s">
         <v>33</v>
       </c>
       <c r="C13" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="D13" t="s">
         <v>18</v>
@@ -3525,7 +3679,7 @@
         <v>23</v>
       </c>
       <c r="N13" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="O13">
         <v>100</v>
@@ -3560,13 +3714,13 @@
     </row>
     <row r="14" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="B14" t="s">
         <v>33</v>
       </c>
       <c r="C14" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="D14" t="s">
         <v>18</v>
@@ -3599,7 +3753,7 @@
         <v>45</v>
       </c>
       <c r="N14" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="O14">
         <v>50</v>
@@ -3634,13 +3788,13 @@
     </row>
     <row r="15" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="B15" t="s">
         <v>33</v>
       </c>
       <c r="C15" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="D15" t="s">
         <v>18</v>
@@ -3673,7 +3827,7 @@
         <v>35</v>
       </c>
       <c r="N15" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="O15">
         <v>65</v>
@@ -3708,13 +3862,13 @@
     </row>
     <row r="16" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="B16" t="s">
         <v>33</v>
       </c>
       <c r="C16" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="D16" t="s">
         <v>18</v>
@@ -3747,7 +3901,7 @@
         <v>35</v>
       </c>
       <c r="N16" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="O16">
         <v>65</v>
@@ -3782,13 +3936,13 @@
     </row>
     <row r="17" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="B17" t="s">
         <v>33</v>
       </c>
       <c r="C17" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="D17" t="s">
         <v>18</v>
@@ -3821,7 +3975,7 @@
         <v>35</v>
       </c>
       <c r="N17" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="O17">
         <v>65</v>
@@ -3856,13 +4010,13 @@
     </row>
     <row r="18" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="B18" t="s">
         <v>33</v>
       </c>
       <c r="C18" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="D18" t="s">
         <v>18</v>
@@ -3871,16 +4025,16 @@
         <v>26</v>
       </c>
       <c r="F18" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="G18" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="H18" t="s">
         <v>21</v>
       </c>
       <c r="I18" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="J18">
         <v>4</v>
@@ -3895,16 +4049,16 @@
         <v>35</v>
       </c>
       <c r="N18" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="O18">
         <v>65</v>
       </c>
       <c r="P18" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="Q18" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="R18" t="s">
         <v>30</v>
@@ -3919,7 +4073,7 @@
         <v>31</v>
       </c>
       <c r="V18" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="W18" t="s">
         <v>33</v>
@@ -3930,13 +4084,13 @@
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="B19" t="s">
         <v>33</v>
       </c>
       <c r="C19" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="D19" t="s">
         <v>18</v>
@@ -3945,16 +4099,16 @@
         <v>26</v>
       </c>
       <c r="F19" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="G19" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="H19" t="s">
         <v>34</v>
       </c>
       <c r="I19" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="J19">
         <v>4</v>
@@ -3969,16 +4123,16 @@
         <v>23</v>
       </c>
       <c r="N19" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="O19">
         <v>100</v>
       </c>
       <c r="P19" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="Q19" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="R19" t="s">
         <v>30</v>
@@ -4004,13 +4158,13 @@
     </row>
     <row r="20" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="B20" t="s">
         <v>33</v>
       </c>
       <c r="C20" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="D20" t="s">
         <v>38</v>
@@ -4043,7 +4197,7 @@
         <v>23</v>
       </c>
       <c r="N20" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="O20">
         <v>100</v>
@@ -4078,13 +4232,13 @@
     </row>
     <row r="21" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="B21" t="s">
         <v>33</v>
       </c>
       <c r="C21" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="D21" t="s">
         <v>38</v>
@@ -4117,7 +4271,7 @@
         <v>23</v>
       </c>
       <c r="N21" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="O21">
         <v>100</v>
@@ -4152,13 +4306,13 @@
     </row>
     <row r="22" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="B22" t="s">
         <v>33</v>
       </c>
       <c r="C22" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="D22" t="s">
         <v>38</v>
@@ -4191,7 +4345,7 @@
         <v>56</v>
       </c>
       <c r="N22" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="O22">
         <v>100</v>
@@ -4226,13 +4380,13 @@
     </row>
     <row r="23" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="B23" t="s">
         <v>33</v>
       </c>
       <c r="C23" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="D23" t="s">
         <v>38</v>
@@ -4265,7 +4419,7 @@
         <v>83</v>
       </c>
       <c r="N23" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="O23">
         <v>65</v>
@@ -4295,6 +4449,154 @@
         <v>33</v>
       </c>
       <c r="X23" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="24" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>174</v>
+      </c>
+      <c r="B24" t="s">
+        <v>33</v>
+      </c>
+      <c r="C24" t="s">
+        <v>141</v>
+      </c>
+      <c r="D24" t="s">
+        <v>18</v>
+      </c>
+      <c r="E24" t="s">
+        <v>26</v>
+      </c>
+      <c r="F24" t="s">
+        <v>90</v>
+      </c>
+      <c r="G24" t="s">
+        <v>104</v>
+      </c>
+      <c r="H24" t="s">
+        <v>21</v>
+      </c>
+      <c r="I24" t="s">
+        <v>107</v>
+      </c>
+      <c r="J24">
+        <v>4</v>
+      </c>
+      <c r="K24">
+        <v>4</v>
+      </c>
+      <c r="L24" t="s">
+        <v>33</v>
+      </c>
+      <c r="M24" t="s">
+        <v>23</v>
+      </c>
+      <c r="N24" t="s">
+        <v>161</v>
+      </c>
+      <c r="O24">
+        <v>100</v>
+      </c>
+      <c r="P24" t="s">
+        <v>105</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>106</v>
+      </c>
+      <c r="R24" t="s">
+        <v>30</v>
+      </c>
+      <c r="S24" t="s">
+        <v>33</v>
+      </c>
+      <c r="T24" t="s">
+        <v>33</v>
+      </c>
+      <c r="U24" t="s">
+        <v>31</v>
+      </c>
+      <c r="V24" t="s">
+        <v>108</v>
+      </c>
+      <c r="W24" t="s">
+        <v>33</v>
+      </c>
+      <c r="X24" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="25" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>175</v>
+      </c>
+      <c r="B25" t="s">
+        <v>33</v>
+      </c>
+      <c r="C25" t="s">
+        <v>141</v>
+      </c>
+      <c r="D25" t="s">
+        <v>18</v>
+      </c>
+      <c r="E25" t="s">
+        <v>26</v>
+      </c>
+      <c r="F25" t="s">
+        <v>90</v>
+      </c>
+      <c r="G25" t="s">
+        <v>113</v>
+      </c>
+      <c r="H25" t="s">
+        <v>21</v>
+      </c>
+      <c r="I25" t="s">
+        <v>107</v>
+      </c>
+      <c r="J25">
+        <v>0</v>
+      </c>
+      <c r="K25">
+        <v>4</v>
+      </c>
+      <c r="L25" t="s">
+        <v>33</v>
+      </c>
+      <c r="M25" t="s">
+        <v>23</v>
+      </c>
+      <c r="N25" t="s">
+        <v>161</v>
+      </c>
+      <c r="O25">
+        <v>100</v>
+      </c>
+      <c r="P25" t="s">
+        <v>105</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>106</v>
+      </c>
+      <c r="R25" t="s">
+        <v>30</v>
+      </c>
+      <c r="S25" t="s">
+        <v>33</v>
+      </c>
+      <c r="T25" t="s">
+        <v>33</v>
+      </c>
+      <c r="U25" t="s">
+        <v>31</v>
+      </c>
+      <c r="V25" t="s">
+        <v>115</v>
+      </c>
+      <c r="W25" t="s">
+        <v>33</v>
+      </c>
+      <c r="X25" t="s">
         <v>33</v>
       </c>
     </row>
@@ -4316,7 +4618,7 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -4343,19 +4645,19 @@
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>16</v>
@@ -4369,7 +4671,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:T22"/>
+  <dimension ref="A1:T24"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -4390,61 +4692,61 @@
   <sheetData>
     <row r="1" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>169</v>
+        <v>178</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>170</v>
+        <v>179</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>172</v>
+        <v>181</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>175</v>
+        <v>184</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>177</v>
+        <v>186</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>11</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>178</v>
+        <v>187</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>180</v>
+        <v>189</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>182</v>
+        <v>191</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>183</v>
+        <v>192</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>184</v>
+        <v>193</v>
       </c>
       <c r="T1" s="1" t="s">
         <v>16</v>
@@ -4452,13 +4754,13 @@
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>185</v>
+        <v>194</v>
       </c>
       <c r="B2" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="C2" t="s">
-        <v>187</v>
+        <v>196</v>
       </c>
       <c r="D2" t="s">
         <v>33</v>
@@ -4509,18 +4811,18 @@
         <v>33</v>
       </c>
       <c r="T2" t="s">
-        <v>188</v>
+        <v>197</v>
       </c>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>185</v>
+        <v>194</v>
       </c>
       <c r="B3" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="C3" t="s">
-        <v>189</v>
+        <v>198</v>
       </c>
       <c r="D3" t="s">
         <v>33</v>
@@ -4576,13 +4878,13 @@
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>185</v>
+        <v>194</v>
       </c>
       <c r="B4" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="C4" t="s">
-        <v>190</v>
+        <v>199</v>
       </c>
       <c r="D4" t="s">
         <v>33</v>
@@ -4638,13 +4940,13 @@
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>191</v>
+        <v>200</v>
       </c>
       <c r="B5" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="C5" t="s">
-        <v>192</v>
+        <v>201</v>
       </c>
       <c r="D5" t="s">
         <v>33</v>
@@ -4653,10 +4955,10 @@
         <v>33</v>
       </c>
       <c r="F5" t="s">
-        <v>193</v>
+        <v>202</v>
       </c>
       <c r="G5" t="s">
-        <v>194</v>
+        <v>203</v>
       </c>
       <c r="H5" t="s">
         <v>33</v>
@@ -4695,18 +4997,18 @@
         <v>33</v>
       </c>
       <c r="T5" t="s">
-        <v>195</v>
+        <v>204</v>
       </c>
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>191</v>
+        <v>200</v>
       </c>
       <c r="B6" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="C6" t="s">
-        <v>196</v>
+        <v>205</v>
       </c>
       <c r="D6" t="s">
         <v>33</v>
@@ -4715,10 +5017,10 @@
         <v>33</v>
       </c>
       <c r="F6" t="s">
-        <v>193</v>
+        <v>202</v>
       </c>
       <c r="G6" t="s">
-        <v>194</v>
+        <v>203</v>
       </c>
       <c r="H6" t="s">
         <v>33</v>
@@ -4762,13 +5064,13 @@
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>191</v>
+        <v>200</v>
       </c>
       <c r="B7" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="C7" t="s">
-        <v>197</v>
+        <v>206</v>
       </c>
       <c r="D7" t="s">
         <v>33</v>
@@ -4777,10 +5079,10 @@
         <v>33</v>
       </c>
       <c r="F7" t="s">
-        <v>193</v>
+        <v>202</v>
       </c>
       <c r="G7" t="s">
-        <v>194</v>
+        <v>203</v>
       </c>
       <c r="H7" t="s">
         <v>33</v>
@@ -4824,13 +5126,13 @@
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>198</v>
+        <v>207</v>
       </c>
       <c r="B8" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="C8" t="s">
-        <v>192</v>
+        <v>201</v>
       </c>
       <c r="D8" t="s">
         <v>33</v>
@@ -4839,10 +5141,10 @@
         <v>33</v>
       </c>
       <c r="F8" t="s">
-        <v>193</v>
+        <v>202</v>
       </c>
       <c r="G8" t="s">
-        <v>199</v>
+        <v>208</v>
       </c>
       <c r="H8" t="s">
         <v>33</v>
@@ -4881,18 +5183,18 @@
         <v>33</v>
       </c>
       <c r="T8" t="s">
-        <v>200</v>
+        <v>209</v>
       </c>
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>198</v>
+        <v>207</v>
       </c>
       <c r="B9" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="C9" t="s">
-        <v>196</v>
+        <v>205</v>
       </c>
       <c r="D9" t="s">
         <v>33</v>
@@ -4901,10 +5203,10 @@
         <v>33</v>
       </c>
       <c r="F9" t="s">
-        <v>193</v>
+        <v>202</v>
       </c>
       <c r="G9" t="s">
-        <v>199</v>
+        <v>208</v>
       </c>
       <c r="H9" t="s">
         <v>33</v>
@@ -4948,13 +5250,13 @@
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>198</v>
+        <v>207</v>
       </c>
       <c r="B10" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="C10" t="s">
-        <v>197</v>
+        <v>206</v>
       </c>
       <c r="D10" t="s">
         <v>33</v>
@@ -4963,10 +5265,10 @@
         <v>33</v>
       </c>
       <c r="F10" t="s">
-        <v>193</v>
+        <v>202</v>
       </c>
       <c r="G10" t="s">
-        <v>199</v>
+        <v>208</v>
       </c>
       <c r="H10" t="s">
         <v>33</v>
@@ -5010,13 +5312,13 @@
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>201</v>
+        <v>210</v>
       </c>
       <c r="B11" t="s">
-        <v>202</v>
+        <v>211</v>
       </c>
       <c r="C11" t="s">
-        <v>203</v>
+        <v>212</v>
       </c>
       <c r="D11" t="s">
         <v>33</v>
@@ -5052,33 +5354,33 @@
         <v>45</v>
       </c>
       <c r="O11" t="s">
-        <v>194</v>
+        <v>203</v>
       </c>
       <c r="P11" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="Q11" t="s">
-        <v>204</v>
+        <v>213</v>
       </c>
       <c r="R11" t="s">
-        <v>205</v>
+        <v>214</v>
       </c>
       <c r="S11" t="s">
-        <v>206</v>
+        <v>215</v>
       </c>
       <c r="T11" t="s">
-        <v>207</v>
+        <v>216</v>
       </c>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>201</v>
+        <v>210</v>
       </c>
       <c r="B12" t="s">
-        <v>202</v>
+        <v>211</v>
       </c>
       <c r="C12" t="s">
-        <v>208</v>
+        <v>217</v>
       </c>
       <c r="D12" t="s">
         <v>33</v>
@@ -5114,19 +5416,19 @@
         <v>45</v>
       </c>
       <c r="O12" t="s">
-        <v>194</v>
+        <v>203</v>
       </c>
       <c r="P12" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="Q12" t="s">
-        <v>204</v>
+        <v>213</v>
       </c>
       <c r="R12" t="s">
-        <v>205</v>
+        <v>214</v>
       </c>
       <c r="S12" t="s">
-        <v>206</v>
+        <v>215</v>
       </c>
       <c r="T12" t="s">
         <v>33</v>
@@ -5134,13 +5436,13 @@
     </row>
     <row r="13" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>201</v>
+        <v>210</v>
       </c>
       <c r="B13" t="s">
-        <v>202</v>
+        <v>211</v>
       </c>
       <c r="C13" t="s">
-        <v>209</v>
+        <v>218</v>
       </c>
       <c r="D13" t="s">
         <v>33</v>
@@ -5176,19 +5478,19 @@
         <v>45</v>
       </c>
       <c r="O13" t="s">
-        <v>194</v>
+        <v>203</v>
       </c>
       <c r="P13" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="Q13" t="s">
-        <v>204</v>
+        <v>213</v>
       </c>
       <c r="R13" t="s">
-        <v>205</v>
+        <v>214</v>
       </c>
       <c r="S13" t="s">
-        <v>206</v>
+        <v>215</v>
       </c>
       <c r="T13" t="s">
         <v>33</v>
@@ -5196,10 +5498,10 @@
     </row>
     <row r="14" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>210</v>
+        <v>219</v>
       </c>
       <c r="B14" t="s">
-        <v>202</v>
+        <v>211</v>
       </c>
       <c r="C14" t="s">
         <v>33</v>
@@ -5238,33 +5540,33 @@
         <v>33</v>
       </c>
       <c r="O14" t="s">
-        <v>194</v>
+        <v>203</v>
       </c>
       <c r="P14" t="s">
-        <v>211</v>
+        <v>220</v>
       </c>
       <c r="Q14" t="s">
-        <v>212</v>
+        <v>221</v>
       </c>
       <c r="R14" t="s">
-        <v>205</v>
+        <v>214</v>
       </c>
       <c r="S14" t="s">
-        <v>206</v>
+        <v>215</v>
       </c>
       <c r="T14" t="s">
-        <v>213</v>
+        <v>222</v>
       </c>
     </row>
     <row r="15" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>214</v>
+        <v>223</v>
       </c>
       <c r="B15" t="s">
-        <v>202</v>
+        <v>211</v>
       </c>
       <c r="C15" t="s">
-        <v>215</v>
+        <v>224</v>
       </c>
       <c r="D15" t="s">
         <v>33</v>
@@ -5300,30 +5602,30 @@
         <v>33</v>
       </c>
       <c r="O15" t="s">
-        <v>194</v>
+        <v>203</v>
       </c>
       <c r="P15" t="s">
-        <v>216</v>
+        <v>225</v>
       </c>
       <c r="Q15" t="s">
-        <v>217</v>
+        <v>226</v>
       </c>
       <c r="R15" t="s">
-        <v>218</v>
+        <v>227</v>
       </c>
       <c r="S15" t="s">
-        <v>219</v>
+        <v>228</v>
       </c>
       <c r="T15" t="s">
-        <v>220</v>
+        <v>229</v>
       </c>
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>221</v>
+        <v>230</v>
       </c>
       <c r="B16" t="s">
-        <v>222</v>
+        <v>231</v>
       </c>
       <c r="C16" t="s">
         <v>33</v>
@@ -5335,16 +5637,16 @@
         <v>95</v>
       </c>
       <c r="F16" t="s">
-        <v>193</v>
+        <v>202</v>
       </c>
       <c r="G16" t="s">
         <v>33</v>
       </c>
       <c r="H16" t="s">
-        <v>223</v>
+        <v>232</v>
       </c>
       <c r="I16" t="s">
-        <v>224</v>
+        <v>233</v>
       </c>
       <c r="J16" t="s">
         <v>33</v>
@@ -5382,10 +5684,10 @@
     </row>
     <row r="17" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>225</v>
+        <v>234</v>
       </c>
       <c r="B17" t="s">
-        <v>222</v>
+        <v>231</v>
       </c>
       <c r="C17" t="s">
         <v>33</v>
@@ -5397,16 +5699,16 @@
         <v>69</v>
       </c>
       <c r="F17" t="s">
-        <v>193</v>
+        <v>202</v>
       </c>
       <c r="G17" t="s">
         <v>33</v>
       </c>
       <c r="H17" t="s">
-        <v>226</v>
+        <v>235</v>
       </c>
       <c r="I17" t="s">
-        <v>224</v>
+        <v>233</v>
       </c>
       <c r="J17" t="s">
         <v>33</v>
@@ -5444,13 +5746,13 @@
     </row>
     <row r="18" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>227</v>
+        <v>236</v>
       </c>
       <c r="B18" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="C18" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="D18" t="s">
         <v>33</v>
@@ -5501,15 +5803,15 @@
         <v>33</v>
       </c>
       <c r="T18" t="s">
-        <v>230</v>
+        <v>239</v>
       </c>
     </row>
     <row r="19" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>227</v>
+        <v>236</v>
       </c>
       <c r="B19" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="C19" t="s">
         <v>33</v>
@@ -5533,13 +5835,13 @@
         <v>33</v>
       </c>
       <c r="J19" t="s">
-        <v>231</v>
+        <v>240</v>
       </c>
       <c r="K19" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
       <c r="L19" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="M19" t="s">
         <v>33</v>
@@ -5568,13 +5870,13 @@
     </row>
     <row r="20" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>233</v>
+        <v>242</v>
       </c>
       <c r="B20" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="C20" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
       <c r="D20" t="s">
         <v>33</v>
@@ -5625,15 +5927,15 @@
         <v>33</v>
       </c>
       <c r="T20" t="s">
-        <v>235</v>
+        <v>244</v>
       </c>
     </row>
     <row r="21" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>233</v>
+        <v>242</v>
       </c>
       <c r="B21" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="C21" t="s">
         <v>33</v>
@@ -5657,13 +5959,13 @@
         <v>33</v>
       </c>
       <c r="J21" t="s">
-        <v>236</v>
+        <v>245</v>
       </c>
       <c r="K21" t="s">
-        <v>237</v>
+        <v>246</v>
       </c>
       <c r="L21" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="M21" t="s">
         <v>33</v>
@@ -5692,13 +5994,13 @@
     </row>
     <row r="22" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>238</v>
+        <v>247</v>
       </c>
       <c r="B22" t="s">
-        <v>239</v>
+        <v>248</v>
       </c>
       <c r="C22" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
       <c r="D22" t="s">
         <v>33</v>
@@ -5749,7 +6051,131 @@
         <v>33</v>
       </c>
       <c r="T22" t="s">
-        <v>241</v>
+        <v>250</v>
+      </c>
+    </row>
+    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>251</v>
+      </c>
+      <c r="B23" t="s">
+        <v>252</v>
+      </c>
+      <c r="C23" t="s">
+        <v>253</v>
+      </c>
+      <c r="D23" t="s">
+        <v>33</v>
+      </c>
+      <c r="E23" t="s">
+        <v>33</v>
+      </c>
+      <c r="F23" t="s">
+        <v>33</v>
+      </c>
+      <c r="G23" t="s">
+        <v>33</v>
+      </c>
+      <c r="H23" t="s">
+        <v>33</v>
+      </c>
+      <c r="I23" t="s">
+        <v>33</v>
+      </c>
+      <c r="J23" t="s">
+        <v>33</v>
+      </c>
+      <c r="K23" t="s">
+        <v>33</v>
+      </c>
+      <c r="L23" t="s">
+        <v>33</v>
+      </c>
+      <c r="M23" t="s">
+        <v>33</v>
+      </c>
+      <c r="N23" t="s">
+        <v>33</v>
+      </c>
+      <c r="O23" t="s">
+        <v>33</v>
+      </c>
+      <c r="P23" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>33</v>
+      </c>
+      <c r="R23" t="s">
+        <v>33</v>
+      </c>
+      <c r="S23" t="s">
+        <v>33</v>
+      </c>
+      <c r="T23" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>251</v>
+      </c>
+      <c r="B24" t="s">
+        <v>252</v>
+      </c>
+      <c r="C24" t="s">
+        <v>255</v>
+      </c>
+      <c r="D24" t="s">
+        <v>33</v>
+      </c>
+      <c r="E24" t="s">
+        <v>33</v>
+      </c>
+      <c r="F24" t="s">
+        <v>33</v>
+      </c>
+      <c r="G24" t="s">
+        <v>33</v>
+      </c>
+      <c r="H24" t="s">
+        <v>33</v>
+      </c>
+      <c r="I24" t="s">
+        <v>33</v>
+      </c>
+      <c r="J24" t="s">
+        <v>33</v>
+      </c>
+      <c r="K24" t="s">
+        <v>33</v>
+      </c>
+      <c r="L24" t="s">
+        <v>33</v>
+      </c>
+      <c r="M24" t="s">
+        <v>33</v>
+      </c>
+      <c r="N24" t="s">
+        <v>33</v>
+      </c>
+      <c r="O24" t="s">
+        <v>33</v>
+      </c>
+      <c r="P24" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>33</v>
+      </c>
+      <c r="R24" t="s">
+        <v>33</v>
+      </c>
+      <c r="S24" t="s">
+        <v>33</v>
+      </c>
+      <c r="T24" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -5771,27 +6197,27 @@
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>242</v>
+        <v>256</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>243</v>
+        <v>257</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>244</v>
+        <v>258</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>245</v>
+        <v>259</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>246</v>
+        <v>260</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>247</v>
+        <v>261</v>
       </c>
       <c r="B2" t="s">
         <v>18</v>
@@ -5811,7 +6237,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>247</v>
+        <v>261</v>
       </c>
       <c r="B3" t="s">
         <v>38</v>
@@ -5831,10 +6257,10 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>248</v>
+        <v>262</v>
       </c>
       <c r="B4" t="s">
-        <v>249</v>
+        <v>263</v>
       </c>
       <c r="C4" t="s">
         <v>33</v>
@@ -5851,10 +6277,10 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>248</v>
+        <v>262</v>
       </c>
       <c r="B5" t="s">
-        <v>250</v>
+        <v>264</v>
       </c>
       <c r="C5" t="s">
         <v>33</v>
@@ -5871,10 +6297,10 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>248</v>
+        <v>262</v>
       </c>
       <c r="B6" t="s">
-        <v>251</v>
+        <v>265</v>
       </c>
       <c r="C6" t="s">
         <v>33</v>
@@ -5897,7 +6323,7 @@
         <v>18</v>
       </c>
       <c r="C7" t="s">
-        <v>252</v>
+        <v>266</v>
       </c>
       <c r="D7" t="s">
         <v>33</v>
@@ -5914,10 +6340,10 @@
         <v>0</v>
       </c>
       <c r="B8" t="s">
-        <v>253</v>
+        <v>267</v>
       </c>
       <c r="C8" t="s">
-        <v>254</v>
+        <v>268</v>
       </c>
       <c r="D8" t="s">
         <v>33</v>
@@ -5937,7 +6363,7 @@
         <v>38</v>
       </c>
       <c r="C9" t="s">
-        <v>255</v>
+        <v>269</v>
       </c>
       <c r="D9" t="s">
         <v>33</v>
@@ -5954,10 +6380,10 @@
         <v>0</v>
       </c>
       <c r="B10" t="s">
-        <v>256</v>
+        <v>270</v>
       </c>
       <c r="C10" t="s">
-        <v>257</v>
+        <v>271</v>
       </c>
       <c r="D10" t="s">
         <v>33</v>
@@ -5971,13 +6397,13 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>258</v>
+        <v>272</v>
       </c>
       <c r="B11" t="s">
         <v>26</v>
       </c>
       <c r="C11" t="s">
-        <v>259</v>
+        <v>273</v>
       </c>
       <c r="D11" t="s">
         <v>33</v>
@@ -5991,13 +6417,13 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>258</v>
+        <v>272</v>
       </c>
       <c r="B12" t="s">
-        <v>260</v>
+        <v>274</v>
       </c>
       <c r="C12" t="s">
-        <v>261</v>
+        <v>275</v>
       </c>
       <c r="D12" t="s">
         <v>33</v>
@@ -6011,13 +6437,13 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>258</v>
+        <v>272</v>
       </c>
       <c r="B13" t="s">
-        <v>262</v>
+        <v>276</v>
       </c>
       <c r="C13" t="s">
-        <v>263</v>
+        <v>277</v>
       </c>
       <c r="D13" t="s">
         <v>33</v>
@@ -6031,13 +6457,13 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>258</v>
+        <v>272</v>
       </c>
       <c r="B14" t="s">
         <v>21</v>
       </c>
       <c r="C14" t="s">
-        <v>264</v>
+        <v>278</v>
       </c>
       <c r="D14" t="s">
         <v>33</v>
@@ -6051,13 +6477,13 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>258</v>
+        <v>272</v>
       </c>
       <c r="B15" t="s">
         <v>34</v>
       </c>
       <c r="C15" t="s">
-        <v>265</v>
+        <v>279</v>
       </c>
       <c r="D15" t="s">
         <v>33</v>
@@ -6071,13 +6497,13 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>258</v>
+        <v>272</v>
       </c>
       <c r="B16" t="s">
         <v>71</v>
       </c>
       <c r="C16" t="s">
-        <v>266</v>
+        <v>280</v>
       </c>
       <c r="D16" t="s">
         <v>33</v>
@@ -6091,13 +6517,13 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>258</v>
+        <v>272</v>
       </c>
       <c r="B17" t="s">
-        <v>267</v>
+        <v>281</v>
       </c>
       <c r="C17" t="s">
-        <v>268</v>
+        <v>282</v>
       </c>
       <c r="D17" t="s">
         <v>33</v>
@@ -6111,16 +6537,16 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>258</v>
+        <v>272</v>
       </c>
       <c r="B18" t="s">
         <v>26</v>
       </c>
       <c r="C18" t="s">
-        <v>269</v>
+        <v>283</v>
       </c>
       <c r="D18" t="s">
-        <v>253</v>
+        <v>267</v>
       </c>
       <c r="E18">
         <v>1</v>
@@ -6146,39 +6572,39 @@
   <sheetData>
     <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>270</v>
+        <v>284</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>271</v>
+        <v>285</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>272</v>
+        <v>286</v>
       </c>
       <c r="B2" t="s">
-        <v>273</v>
+        <v>287</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>274</v>
+        <v>288</v>
       </c>
       <c r="B3" t="s">
-        <v>275</v>
+        <v>289</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>276</v>
+        <v>290</v>
       </c>
       <c r="B4" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>244</v>
+        <v>258</v>
       </c>
       <c r="B5" t="s">
         <v>33</v>
@@ -6186,7 +6612,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>277</v>
+        <v>291</v>
       </c>
       <c r="B6" t="s">
         <v>33</v>
@@ -6194,23 +6620,23 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>278</v>
+        <v>292</v>
       </c>
       <c r="B7" t="s">
-        <v>279</v>
+        <v>293</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>280</v>
+        <v>294</v>
       </c>
       <c r="B8" t="s">
-        <v>281</v>
+        <v>295</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>282</v>
+        <v>296</v>
       </c>
       <c r="B9" t="s">
         <v>33</v>
@@ -6218,7 +6644,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>283</v>
+        <v>297</v>
       </c>
       <c r="B10" t="s">
         <v>33</v>
@@ -6226,7 +6652,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>284</v>
+        <v>298</v>
       </c>
       <c r="B11" t="s">
         <v>33</v>

</xml_diff>

<commit_message>
Examples: every person has a first and a last name
Assisted by Claude Sonnet 5.5 (Anthropic).
</commit_message>
<xml_diff>
--- a/apps/web/public/examples/example-with-constraint-rules.xlsx
+++ b/apps/web/public/examples/example-with-constraint-rules.xlsx
@@ -118,7 +118,7 @@
     <t>Musical Patterns II</t>
   </si>
   <si>
-    <t>Kim</t>
+    <t>Kim Mockup</t>
   </si>
   <si>
     <t>Lecture</t>
@@ -265,10 +265,10 @@
     <t>Introduction to Behavioral Dynamics</t>
   </si>
   <si>
-    <t>Lee</t>
-  </si>
-  <si>
-    <t>Lee's two sections are not back to back</t>
+    <t>Lee Standin</t>
+  </si>
+  <si>
+    <t>Lee Standin's two sections are not back to back</t>
   </si>
   <si>
     <t>C</t>
@@ -355,7 +355,7 @@
     <t>Network Optimization</t>
   </si>
   <si>
-    <t>Kim teaches three in a row on MWF</t>
+    <t>Kim Mockup teaches three in a row on MWF</t>
   </si>
   <si>
     <t>318</t>
@@ -736,7 +736,7 @@
     <t>At least one section must meet within the evening hours.</t>
   </si>
   <si>
-    <t>Kim: at most two classes in a row</t>
+    <t>Kim Mockup: at most two classes in a row</t>
   </si>
   <si>
     <t>consecutive</t>
@@ -748,7 +748,7 @@
     <t>20</t>
   </si>
   <si>
-    <t>Lee: at least two classes in a row</t>
+    <t>Lee Standin: at least two classes in a row</t>
   </si>
   <si>
     <t>atLeast</t>
@@ -913,7 +913,7 @@
     <t>Export Time</t>
   </si>
   <si>
-    <t>14:23:18</t>
+    <t>15:09:00</t>
   </si>
   <si>
     <t>Academic Year</t>

</xml_diff>